<commit_message>
feat : LMS upgrade
</commit_message>
<xml_diff>
--- a/Dinduction.Web/wwwroot/Template.xlsx
+++ b/Dinduction.Web/wwwroot/Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\Rian\Code .net\Training\Training\Training.Web\AdminLTE\dist\img\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rian.ardana\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2B34E1-D0A7-4C21-8E56-96EB11B709BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B20ADA-40BA-4CA9-BE43-94C56EA18C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{841BC58D-0D10-485D-B98A-11D7A0F72C54}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>NO BADGE</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>DEPARTMENT</t>
+  </si>
+  <si>
+    <t>Training Type (I/R)</t>
   </si>
 </sst>
 </file>
@@ -425,14 +428,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8099629-EAC7-404C-AC43-273590126296}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,6 +447,9 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>